<commit_message>
test: all tests passing, integration verified
</commit_message>
<xml_diff>
--- a/data/Matriz_Normativa_IA_Educacion_LATAM.xlsx
+++ b/data/Matriz_Normativa_IA_Educacion_LATAM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30125"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tecmx-my.sharepoint.com/personal/a00834778_tec_mx/Documents/Desktop/Carlos Auquilla/Proyectos/GENIAL/GENIAL_dev/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DEF93B8B-1B75-490B-94A3-E0F7B496BF87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="428" documentId="8_{DEF93B8B-1B75-490B-94A3-E0F7B496BF87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{350EF929-F841-4D67-802D-87771D8B7F4B}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1595" uniqueCount="529">
   <si>
     <t>Investigador</t>
   </si>
@@ -1109,6 +1109,434 @@
     <t>Establece la creación del 'Consejo Coordinador de Inteligencia Artificial' en la UNAM, con el objetivo de potenciar las capacidades institucionales en IA y fortalecer la autonomía tecnológica de la Universidad.</t>
   </si>
   <si>
+    <t>Inteligencia Artificial y la Imaginación Humana: Una Investigación Ética</t>
+  </si>
+  <si>
+    <t>https://www.ipn.mx/assets/files/innovacion/docs/Docencia-politecnica/Docencia-politecnica-24/inteligencia-artificial-y-la-inaginacion-humana.pdf</t>
+  </si>
+  <si>
+    <t>Documento académico no vinculante. Analiza implicaciones éticas de IA generativa en creatividad, formación docente y educación superior. Discute sesgos, propiedad intelectual, dependencia tecnológica y complementariedad humano-IA.</t>
+  </si>
+  <si>
+    <t>Guía de uso de inteligencia artificial generativa en la evaluación educativa en el posgrado</t>
+  </si>
+  <si>
+    <t>https://www.pdcb.unam.mx/documentos/alumnos/guia-de-uso-de-inteligencia-artificial-generativa-en-evaluacion-educativa-en-el-posgrado.pdf?ui=1409252254</t>
+  </si>
+  <si>
+    <t>Documento institucional de referencia para uso ético y pedagógico de IA generativa en evaluación de posgrado. Incluye principios de integridad académica, alfabetización en IA, evaluación híbrida, uso responsable de LLMs, sesgos algorítmicos y lineamientos para docentes y estudiantes. Promueve enfoque humanista y evaluación crítica del uso de IA.</t>
+  </si>
+  <si>
+    <t>Pautas para hacer uso de la Inteligencia Artificial en la Formación Docente Universitaria</t>
+  </si>
+  <si>
+    <t>https://cfop.ceide.unam.mx/wp-content/uploads/2025/06/Conferencia-Pautas-para-hacer-uso-de-la-IA-en-la-formacion-docente-universitaria.pdf</t>
+  </si>
+  <si>
+    <t>Documento presentado en el IV Seminario Internacional Educación y TAC. Incluye pautas institucionales para uso ético de IA, programas de formación docente, microtalleres y adopción transversal de IA generativa en educación superior. Evidencia institucionalización progresiva de IA en la UNAM.</t>
+  </si>
+  <si>
+    <t>Relevancia de la Inteligencia Artificial en la educación</t>
+  </si>
+  <si>
+    <t>https://www.zaragoza.unam.mx/wp-content/2023/Publicaciones/libros/csociales/Relevancia_IA_educacion.pdf</t>
+  </si>
+  <si>
+    <t>Compilación institucional revisada por pares sobre IA en educación. Incluye revisión sistemática sobre LLMs en educación latinoamericana, ética, evaluación, gestión académica y formación profesional. Refleja madurez institucional y adopción formal de IA educativa en UNAM.</t>
+  </si>
+  <si>
+    <t>Políticas de uso de Inteligencia Artificial para trabajos académicos</t>
+  </si>
+  <si>
+    <t>https://www.economia.unam.mx/profesores/eloria/index_htm_files/Uso%20de%20IA.pdf</t>
+  </si>
+  <si>
+    <t>Define usos permitidos y prohibidos de IA generativa en trabajos académicos, incorpora declaración obligatoria de uso IA y mecanismos de sanción. Representa regulación institucional madura de IA académica.</t>
+  </si>
+  <si>
+    <t>La Inteligencia Artificial Generativa (IAGEN) en el profesorado y estudiantado de la UNAM. Retos y prospectivas</t>
+  </si>
+  <si>
+    <t>https://www.ceide.unam.mx/wp-content/uploads/2025/08/IAGen_UNAM_2025.pdf</t>
+  </si>
+  <si>
+    <t>Documento institucional oficial que diagnostica el uso de IA generativa en educación superior UNAM. No establece regulación obligatoria, pero sí orientaciones estratégicas, éticas y pedagógicas. Referencia explícita al proyecto institucional “Desarrollo de la IAGen en la docencia universitaria” del PDI 2023–2027.</t>
+  </si>
+  <si>
+    <t>Derechos digitales y la sexta generación: acceso, privacidad y libertad en el ciberespacio</t>
+  </si>
+  <si>
+    <t>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;opi=89978449&amp;url=https://revistas.juridicas.unam.mx/index.php/hechos-y-derechos/article/view/19934/19951&amp;ved=2ahUKEwjKp6in-tSUAxV9fTABHSpdFtI4FBAWegQIMBAB&amp;usg=AOvVaw3ajc17fzIwcN8MDw3wACsR</t>
+  </si>
+  <si>
+    <t>Artículo académico-jurídico sobre derechos digitales, privacidad, IA ética y gobernanza del ciberespacio. No constituye normativa vinculante ni política institucional, pero refleja tendencias doctrinales y preocupaciones regulatorias emergentes en México.</t>
+  </si>
+  <si>
+    <t>Recomendaciones sobre el uso de materiales explícitos y/o sensibles en actividades docentes en la ENaCiF</t>
+  </si>
+  <si>
+    <t>https://www.enacif.unam.mx/wp-content/uploads/2025/05/Sintesis-Recomendaciones-sobre-el-uso-de-Materiales-Explicitos-y_o-Sensibles-en-actividades-docentes-en-la-ENaCiF.pdf</t>
+  </si>
+  <si>
+    <t>Documento institucional que regula el manejo ético de materiales sensibles en actividades docentes. Incluye referencia explícita al posible uso de imágenes generadas mediante inteligencia artificial y establece principios de inclusión, consentimiento, privacidad y enfoque informado sobre trauma.</t>
+  </si>
+  <si>
+    <t>Plan de Desarrollo IIMAS-UNAM 2024-2028</t>
+  </si>
+  <si>
+    <t>https://www.iimas.unam.mx/wp-content/uploads/2025/04/Plan-de-Desarrollo-IIMAS-2024_2028-v1.pdf</t>
+  </si>
+  <si>
+    <t>El documento plantea la creación formal de “Principios IIMAS para una IA Ética, Responsable y Sostenible”, incluyendo aprobación institucional, regulación del actuar académico, capacitación docente y uso de IA generativa en educación. Constituye evidencia de gobernanza institucional emergente sobre IA en educación superior.</t>
+  </si>
+  <si>
+    <t>Políticas Educativas: Lecciones del IFE Conference 2024</t>
+  </si>
+  <si>
+    <t>Fecha no disponible: inferida
+por contexto del año 2024</t>
+  </si>
+  <si>
+    <t>https://tec.mx/sites/default/files/repositorio/ife/pdf/politicas-educativas-ife-tec-de-monterrey.pdf?srsltid=AfmBOop0NBuvTlnWsQNr0jjulBXKVddrSclv1GBNCc1pGB9TZUS7Cckj</t>
+  </si>
+  <si>
+    <t>Documento estratégico sobre IA en educación, alfabetización IA, riesgos éticos, desinformación, privacidad y regulación. Referencia marcos UNESCO y tendencias globales de gobernanza educativa.</t>
+  </si>
+  <si>
+    <t>Congreso Internacional de Inteligencia Artificial: potencial, retos y oportunidades para México</t>
+  </si>
+  <si>
+    <t>https://www.ipn.mx/assets/files/imageninstitucional/docs/identidad/2025/05/uso-ia.pdf</t>
+  </si>
+  <si>
+    <t>Documento institucional sobre gobernanza, ética, protección de datos y uso educativo de IA. No constituye regulación vinculante.</t>
+  </si>
+  <si>
+    <t>Uso personal y académico de inteligencia artificial en estudiantes universitarios: estudio exploratorio</t>
+  </si>
+  <si>
+    <t>30/03/2025</t>
+  </si>
+  <si>
+    <t>https://apertura.cugdl.udg.mx/index.php/apertura/article/view/2604</t>
+  </si>
+  <si>
+    <t>Estudio empírico sobre adopción real de IA en educación superior mexicana. Identifica uso masivo de ChatGPT y otras IA, ausencia de acceso institucional formal, necesidad de regulación ética y vacíos de gobernanza universitaria. Útil como evidencia contextual de madurez y barreras de adopción.</t>
+  </si>
+  <si>
+    <t>Inteligencia Artificial Generativa: Enfoques Prácticos para Docentes (Edu Book)</t>
+  </si>
+  <si>
+    <t>https://observatorio.tec.mx/wp-content/uploads/2025/07/EDU-BOOK_IA-GENERATIVA_V6.pdf</t>
+  </si>
+  <si>
+    <t>Edu book realizado para reportar el observatorio realizado por el instituto por el futuro de la educación del Tecnológico de Monterrey. Una herramienta enfocada en la implementación práctica de la IA y sus implicaciones éticas</t>
+  </si>
+  <si>
+    <t>Guía para el Uso Ético y Responsable de la Inteligencia Artificial Generativa en Entornos Digitales para el Aprendizaje</t>
+  </si>
+  <si>
+    <t>Integra el uso de la Inteligencia Artificial con el cóidgio de ética de la institución y sus regulaciones disciplinarias</t>
+  </si>
+  <si>
+    <t>Principios de acción para un uso ético y crítico de la IAG en la educación superior mexicana</t>
+  </si>
+  <si>
+    <t>https://www.gob.mx/cms/uploads/attachment/file/1071410/ENIAG2025_PRINCIPIOS.pdf</t>
+  </si>
+  <si>
+    <t>Define 10 principios como un marco de trabajo para la agenda de Educación Superior y solicita establecer lineamientos institucionales claros para el usoético, crítico y con propóstio dentro de las instituciones.</t>
+  </si>
+  <si>
+    <t>Observatorio Interinstitucional de Inteligencia Artificial en la Educación Superior en México: Documento Fundacional</t>
+  </si>
+  <si>
+    <t>ANUIES, FIMPES, UNAM, UAM, UPN, Santander</t>
+  </si>
+  <si>
+    <t>https://observatorio-ia.org/OIIAES.pdf</t>
+  </si>
+  <si>
+    <t>Marco de trabajo colaborativo interinstitucional para monitorear el impacto de la Inteligencia Artificial y generar una política pública. Su objetivo es monitorear las prácticas de integración de la IA en la educación superior sistematizando y
+evaluando su integración en este nivel educativo</t>
+  </si>
+  <si>
+    <t>México: evaluación del estadío de preparación de la inteligencia artificial</t>
+  </si>
+  <si>
+    <t>https://unesdoc.unesco.org/ark:/48223/pf0000390568</t>
+  </si>
+  <si>
+    <t>Perfil país de UNESCO que funciona como índice del ecosistema de IA en México, no como norma vinculante. Sirve para contextualizar políticas universitarias y ubicar documentos nacionales. Su límite es que resume información y no fija obligaciones legales. Conviene incluirlo solo como fuente contextual.</t>
+  </si>
+  <si>
+    <t>Lineamientos para el uso de herramientas de inteligencia artificial en CETYS Universidad</t>
+  </si>
+  <si>
+    <t>https://www.cetys.mx/wp-content/uploads/2024/04/Comunicado-Vicerrectoria-Academica-IA.pdf</t>
+  </si>
+  <si>
+    <t>Establece pautas para el uso de herramientas de IA en actividades académicas, incluyendo condiciones sobre "propiedad intelectual" y "plagio". Promueve la "alfabetización en IA" como parte de las competencias educativas en CETYS Universidad.</t>
+  </si>
+  <si>
+    <t>Guía en inteligencia artificial: grupo de trabajo de alfabetización en IA</t>
+  </si>
+  <si>
+    <t>Establece un marco para la 'alfabetización en inteligencia artificial' en CETYS Universidad, sugiriendo elementos básicos de conocimiento y terminología. Se deriva de los 'Lineamientos para el uso de herramientas de inteligencia artificial' emitidos en octubre de 2023.</t>
+  </si>
+  <si>
+    <t>Maestría en Audio y la Industria del Entretenimiento Digital con Certificación en Negocios del Entretenimiento</t>
+  </si>
+  <si>
+    <t>Fermatta</t>
+  </si>
+  <si>
+    <t>https://www.fermatta.edu.mx/planes-educativos-mae/maestr%C3%ADa-en-audio-y-la-industria-del-entretenimiento-digital-con-certificaci%C3%B3n-en-negocios-del-entretenimiento</t>
+  </si>
+  <si>
+    <t>Establece un programa académico que incluye 'Herramientas de Inteligencia Artificial para la Creación de Música' en varios semestres. Promueve el uso de tecnología avanzada en la producción musical, integrando IA como parte fundamental de la formación profesional en la industria del entretenimiento.</t>
+  </si>
+  <si>
+    <t>Diseño de materiales digitales</t>
+  </si>
+  <si>
+    <t>Secretaría de Educación Pública</t>
+  </si>
+  <si>
+    <t>01/01/2023</t>
+  </si>
+  <si>
+    <t>http://www.sev.gob.mx/educacion-normal/curricular/wp-content/uploads/sites/14/2026/03/ENJE_LEP_6o_Diseno-de-materiales-Digitales.pdf</t>
+  </si>
+  <si>
+    <t>Establece el desarrollo de habilidades para diseñar materiales digitales educativos e incorpora la formación en el uso pedagógico, crítico y ético de herramientas basadas en 'inteligencia artificial'. Este curso busca preparar a los futuros educadores para crear recursos inclusivos y accesibles en entornos preescolares.</t>
+  </si>
+  <si>
+    <t>Maestría en Audio y la Industria del Entretenimiento Digital con Certificación en Mezcla</t>
+  </si>
+  <si>
+    <t>Centro Universitario de Música Fermatta</t>
+  </si>
+  <si>
+    <t>https://www.fermatta.edu.mx/planes-educativos-mae/maestr%C3%ADa-en-audio-y-la-industria-del-entretenimiento-digital-con-certificaci%C3%B3n-en-mezcla</t>
+  </si>
+  <si>
+    <t>Establece un programa académico que incluye 'Herramientas de Inteligencia Artificial para la Creación de Música' en varios semestres. Proporciona formación en técnicas de mezcla y producción musical, integrando aplicaciones avanzadas de IA en la educación musical.</t>
+  </si>
+  <si>
+    <t>Ley General de Humanidades, Ciencia, Tecnología e Innovación</t>
+  </si>
+  <si>
+    <t>Gobierno de México</t>
+  </si>
+  <si>
+    <t>https://sipot.ciateq.mx/planeacion/29%20XXIX%20INFORMES/Informe_In_Extenso_2023_ene_jun.pdf.pdf</t>
+  </si>
+  <si>
+    <t>Establece la evaluación de la gestión en el marco del Programa Institucional y menciona la 'evaluación de su gestión' como parte de las nuevas disposiciones. Aunque no se centra en IA, su aplicación puede influir en la regulación de tecnologías emergentes en el ámbito educativo.</t>
+  </si>
+  <si>
+    <t>Código de Ética e Integridad para un Buen Gobierno en la Administración Pública Federal</t>
+  </si>
+  <si>
+    <t>Secretaría Anticorrupción y Buen Gobierno</t>
+  </si>
+  <si>
+    <t>18/11/2025</t>
+  </si>
+  <si>
+    <t>https://www.cibnor.gob.mx/files/admon/DOF_CODIGO_ETICA_APF_2025.pdf</t>
+  </si>
+  <si>
+    <t>Establece principios de 'ética e integridad' para la administración pública. Aunque no menciona IA directamente, su enfoque en la ética es relevante para la gobernanza de tecnologías emergentes en el sector educativo.</t>
+  </si>
+  <si>
+    <t>Ley General en Materia de Humanidades, Ciencias, Tecnologías e Innovación</t>
+  </si>
+  <si>
+    <t>CIATEC, A.C., CENTRO DE INNOVACIÓN APLICADA EN TECNOLOGÍAS COMPETITIVAS</t>
+  </si>
+  <si>
+    <t>Mención breve</t>
+  </si>
+  <si>
+    <t>08/05/2023</t>
+  </si>
+  <si>
+    <t>https://www.ciatec.mx/archivos/98bafc961336f547dcd60e17270c6c5b.pdf</t>
+  </si>
+  <si>
+    <t>Establece un marco normativo para la promoción de 'Ciencias, Tecnologías e Innovación', incluyendo aspectos relacionados con la inteligencia artificial. Aunque no se centra exclusivamente en IA, su relevancia para la gobernanza de tecnologías emergentes es significativa.</t>
+  </si>
+  <si>
+    <t>Lineamientos Complementarios para la Maestría en Ciencias con Orientación en Robótica</t>
+  </si>
+  <si>
+    <t>Centro de Investigación en Matemáticas, A. C. (Cimat)</t>
+  </si>
+  <si>
+    <t>https://mcr.cimat.mx/es/Lineamientos_MCR</t>
+  </si>
+  <si>
+    <t>Regula el funcionamiento de la Maestría en Ciencias con Orientación en Robótica, incluyendo la formación en 'inteligencia artificial' y su interacción con la robótica. Establece lineamientos para la calidad académica y la estructura del programa de posgrado.</t>
+  </si>
+  <si>
+    <t>SIP-30</t>
+  </si>
+  <si>
+    <t>01/01/2021</t>
+  </si>
+  <si>
+    <t>https://www.cic.ipn.mx/doc/MCyTIAyCD/5-Opt-IA-explicativa-interpretable.pdf</t>
+  </si>
+  <si>
+    <t>Establece los lineamientos para la unidad de aprendizaje 'Inteligencia Artificial Explicativa e Interpretable', incluyendo objetivos de aprendizaje y competencias específicas en el ámbito de la IA. Define la estructura curricular y los requisitos para la maestría en Ciencia y Tecnología de Inteligencia Artificial y Ciencia de Datos.</t>
+  </si>
+  <si>
+    <t>Inteligencia Artificial Explicable</t>
+  </si>
+  <si>
+    <t>26/07/2023</t>
+  </si>
+  <si>
+    <t>https://www.cic.ipn.mx/doc/DCC/15.%20Inteligencia-Artificial-Explicable-Registrada.pdf</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para la unidad de aprendizaje 'Inteligencia Artificial Explicable', incluyendo conceptos de 'transparencia' y 'explicabilidad' en IA. Define aprendizajes y habilidades que los estudiantes deben demostrar, promoviendo la responsabilidad y la ética en el uso de IA.</t>
+  </si>
+  <si>
+    <t>Política de uso de IA</t>
+  </si>
+  <si>
+    <t>CIATEJ</t>
+  </si>
+  <si>
+    <t>https://revistaenfoques.ciatej.mx/index.php/revistaenfoques/politica_uso_de_IA</t>
+  </si>
+  <si>
+    <t>Establece directrices para el 'uso de inteligencia artificial' en el contexto institucional. Define el empleo de herramientas digitales basadas en modelos generativos, orientando su aplicación en la educación superior.</t>
+  </si>
+  <si>
+    <t>Programa de Trabajo - CIATEC</t>
+  </si>
+  <si>
+    <t>CIATEC</t>
+  </si>
+  <si>
+    <t>https://www.ciatec.mx/archivos/fbbd14366497df3a41a3023121745292.pdf</t>
+  </si>
+  <si>
+    <t>Establece un programa de trabajo que incluye la 'inteligencia artificial' como parte de las especialidades en el posgrado, promoviendo la formación de recursos humanos con capacidad de respuesta a necesidades sociales e industriales. Se enfoca en la vinculación con sectores educativos y tecnológicos para democratizar el conocimiento.</t>
+  </si>
+  <si>
+    <t>PLAN DE TRABAJO - CIATEC</t>
+  </si>
+  <si>
+    <t>https://www.ciatec.mx/archivos/04ae246e577be2fd8cd2b915aba3c9c3.pdf</t>
+  </si>
+  <si>
+    <t>Impulsa la 'investigación y desarrollo tecnológico' en áreas como 'inteligencia artificial' y 'robótica'. Establece colaboración con empresas e instituciones para fomentar políticas que protejan el medio ambiente y promuevan la sostenibilidad.</t>
+  </si>
+  <si>
+    <t>7.1.7 Coordinación de Datos y Analítica</t>
+  </si>
+  <si>
+    <t>Dirección de Innovación y Desarrollo Tecnológico</t>
+  </si>
+  <si>
+    <t>https://reposipot.imss.gob.mx/organizacion/UP/CNMEMPRH/CTOMP/2025/F_III_Atribuciones-Funciones/NC/9_DIDT/7.1.7%20Coord.%20de%20Datos%20y%20Analitica_DIDT.pdf</t>
+  </si>
+  <si>
+    <t>Coordina la implementación de 'políticas, lineamientos y criterios' en materia de 'inteligencia artificial' y 'analítica de datos'. Establece procedimientos para la transferencia de conocimientos y supervisa el diseño de herramientas tecnológicas relacionadas con la IA.</t>
+  </si>
+  <si>
+    <t>Declaración sobre Inteligencia Artificial</t>
+  </si>
+  <si>
+    <t>Revista Médica del IMSS</t>
+  </si>
+  <si>
+    <t>https://revistamedica.imss.gob.mx/index.php/revista_medica/IA</t>
+  </si>
+  <si>
+    <t>Establece criterios editoriales para el uso responsable de IA en el ámbito biomédico, incluyendo 'transparencia', 'responsabilidad humana' y 'protección de datos'. Regula el uso de herramientas de IA en la elaboración y revisión de manuscritos, enfatizando la supervisión humana y la confidencialidad.</t>
+  </si>
+  <si>
+    <t>Uso de la Inteligencia Artificial para disminuir los costos</t>
+  </si>
+  <si>
+    <t>Colegio de Contadores Públicos de Guadalajara Jalisco</t>
+  </si>
+  <si>
+    <t>01/06/2024</t>
+  </si>
+  <si>
+    <t>https://ccpg.org.mx/wp-content/uploads/2024/06/Vision_contable_mayo_2024.pdf</t>
+  </si>
+  <si>
+    <t>Establece directrices sobre el 'Uso de la Inteligencia Artificial para disminuir los costos' en el ámbito contable. Proporciona un enfoque técnico que puede influir en la implementación de IA en procesos educativos y administrativos.</t>
+  </si>
+  <si>
+    <t>Política de supervisión ética</t>
+  </si>
+  <si>
+    <t>El Colegio de la Frontera Norte</t>
+  </si>
+  <si>
+    <t>https://ojs.colef.mx/index.php/fronteranorte/politica_de_supervision_etica</t>
+  </si>
+  <si>
+    <t>Regula el uso de herramientas de inteligencia artificial bajo los 'lineamientos establecidos por la Secretaría de Ciencia, Humanidades, Tecnología'. Establece principios éticos para su implementación en el ámbito educativo.</t>
+  </si>
+  <si>
+    <t>4º CONCURSO DE CREATIVIDAD DIGITAL 2026</t>
+  </si>
+  <si>
+    <t>Colegio Alemán</t>
+  </si>
+  <si>
+    <t>01/01/2026</t>
+  </si>
+  <si>
+    <t>https://humboldt.edu.mx/creatividad-digital/wp-content/uploads/2026/01/Convocatoria-4-Concurso-de-Creatividad-Digital-Primaria.pdf</t>
+  </si>
+  <si>
+    <t>Establece lineamientos para la participación en un concurso de creatividad digital, prohibiendo el 'uso de inteligencia artificial' y plantillas prediseñadas en los proyectos. Promueve la originalidad y la asesoría docente en la creación de productos multimedia.</t>
+  </si>
+  <si>
+    <t>Plan de Acción_G3.14_Anexo_Entregar</t>
+  </si>
+  <si>
+    <t>https://soporte.enesmorelia.unam.mx/respuesta-pliegos-petitorios/doc/3/3.14_Anexo.pdf</t>
+  </si>
+  <si>
+    <t>Establece la oferta de cursos relacionados con 'ética e inteligencia artificial' y 'herramientas de Inteligencia Artificial para Docentes'. Refleja un interés institucional por integrar la IA en la formación docente y la práctica educativa.</t>
+  </si>
+  <si>
+    <t>Política de uso IA</t>
+  </si>
+  <si>
+    <t>Frontera Norte</t>
+  </si>
+  <si>
+    <t>https://fronteranorte.colef.mx/index.php/fronteranorte/politica_de_IA</t>
+  </si>
+  <si>
+    <t>Exige 'transparencia total' en el uso de herramientas de inteligencia artificial durante la elaboración de manuscritos. Establece principios éticos para el uso de IA en el contexto académico.</t>
+  </si>
+  <si>
+    <t>Maestría: Asuntos Políticos y Políticas Públicas</t>
+  </si>
+  <si>
+    <t>Colegio de San Luis</t>
+  </si>
+  <si>
+    <t>https://www.colsan.edu.mx/arch/mappp/MAPPP-10a_2026-28.pdf</t>
+  </si>
+  <si>
+    <t>Prohíbe el uso de 'Inteligencia Artificial generativa' en la elaboración de anteproyectos. Establece lineamientos para la admisión a la maestría en asuntos políticos y políticas públicas, incluyendo la detección de plagio.</t>
+  </si>
+  <si>
     <t>Brasil</t>
   </si>
   <si>
@@ -1209,9 +1637,6 @@
   </si>
   <si>
     <t>Derrogada</t>
-  </si>
-  <si>
-    <t>Mención breve</t>
   </si>
 </sst>
 </file>
@@ -1222,7 +1647,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="165" formatCode="dd\.mm\.yyyy;@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1255,6 +1680,14 @@
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1321,10 +1754,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1356,8 +1790,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1658,7 +2098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M106"/>
+  <dimension ref="A1:M135"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="16.140625" customWidth="1"/>
@@ -4629,14 +5069,14 @@
         <v>43</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="15">
+    <row r="73" spans="1:13" ht="30.75">
       <c r="A73" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="C73" s="12" t="s">
         <v>315</v>
       </c>
       <c r="D73" s="3" t="s">
@@ -5039,343 +5479,1846 @@
         <v>43</v>
       </c>
     </row>
-    <row r="83" spans="1:13" ht="15">
-      <c r="A83" s="3"/>
-      <c r="B83" s="3"/>
-      <c r="C83" s="3"/>
-      <c r="D83" s="3"/>
-      <c r="E83" s="3"/>
-      <c r="F83" s="3"/>
-      <c r="G83" s="3"/>
-      <c r="I83" s="3"/>
-      <c r="J83" s="6"/>
-      <c r="K83" s="3"/>
-      <c r="L83" s="3"/>
-      <c r="M83" s="3"/>
-    </row>
-    <row r="84" spans="1:13" ht="15">
-      <c r="A84" s="3"/>
-      <c r="B84" s="3"/>
-      <c r="C84" s="3"/>
-      <c r="D84" s="3"/>
-      <c r="E84" s="3"/>
-      <c r="F84" s="3"/>
-      <c r="G84" s="3"/>
-      <c r="H84" s="3"/>
-      <c r="I84" s="3"/>
-      <c r="J84" s="6"/>
-      <c r="K84" s="3"/>
-      <c r="L84" s="3"/>
-      <c r="M84" s="3"/>
-    </row>
-    <row r="85" spans="1:13" ht="15">
-      <c r="A85" s="3"/>
-      <c r="B85" s="3"/>
-      <c r="C85" s="3"/>
-      <c r="D85" s="3"/>
-      <c r="E85" s="3"/>
-      <c r="F85" s="3"/>
-      <c r="G85" s="3"/>
-      <c r="H85" s="3"/>
-      <c r="I85" s="3"/>
-      <c r="J85" s="6"/>
-      <c r="K85" s="3"/>
-      <c r="L85" s="3"/>
-      <c r="M85" s="3"/>
-    </row>
-    <row r="86" spans="1:13" ht="15">
-      <c r="A86" s="3"/>
-      <c r="B86" s="3"/>
-      <c r="C86" s="3"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
-      <c r="F86" s="3"/>
-      <c r="G86" s="3"/>
-      <c r="H86" s="3"/>
-      <c r="I86" s="3"/>
-      <c r="J86" s="6"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="3"/>
-      <c r="M86" s="3"/>
-    </row>
-    <row r="87" spans="1:13" ht="15">
-      <c r="A87" s="3"/>
-      <c r="B87" s="3"/>
-      <c r="C87" s="3"/>
-      <c r="D87" s="3"/>
-      <c r="E87" s="3"/>
-      <c r="F87" s="3"/>
-      <c r="G87" s="3"/>
-      <c r="H87" s="3"/>
-      <c r="I87" s="3"/>
-      <c r="J87" s="6"/>
-      <c r="K87" s="3"/>
-      <c r="L87" s="3"/>
-      <c r="M87" s="3"/>
-    </row>
-    <row r="88" spans="1:13" ht="15">
-      <c r="A88" s="3"/>
-      <c r="B88" s="3"/>
-      <c r="C88" s="3"/>
-      <c r="D88" s="3"/>
-      <c r="E88" s="3"/>
-      <c r="F88" s="3"/>
-      <c r="G88" s="3"/>
-      <c r="H88" s="3"/>
-      <c r="I88" s="3"/>
-      <c r="J88" s="6"/>
-      <c r="K88" s="3"/>
-      <c r="L88" s="3"/>
-      <c r="M88" s="3"/>
-    </row>
-    <row r="89" spans="1:13" ht="15">
-      <c r="A89" s="3"/>
-      <c r="B89" s="3"/>
-      <c r="C89" s="3"/>
-      <c r="D89" s="3"/>
-      <c r="E89" s="3"/>
-      <c r="F89" s="3"/>
-      <c r="G89" s="3"/>
-      <c r="H89" s="3"/>
-      <c r="I89" s="3"/>
-      <c r="J89" s="6"/>
-      <c r="K89" s="3"/>
-      <c r="L89" s="3"/>
-      <c r="M89" s="3"/>
-    </row>
-    <row r="90" spans="1:13" ht="15">
-      <c r="A90" s="3"/>
-      <c r="B90" s="3"/>
-      <c r="C90" s="3"/>
-      <c r="D90" s="3"/>
-      <c r="E90" s="3"/>
-      <c r="F90" s="3"/>
-      <c r="G90" s="3"/>
-      <c r="H90" s="3"/>
-      <c r="I90" s="3"/>
-      <c r="J90" s="6"/>
-      <c r="K90" s="3"/>
-      <c r="L90" s="3"/>
-      <c r="M90" s="3"/>
-    </row>
-    <row r="91" spans="1:13" ht="15">
-      <c r="A91" s="3"/>
-      <c r="B91" s="3"/>
-      <c r="C91" s="3"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="3"/>
-      <c r="F91" s="3"/>
-      <c r="G91" s="3"/>
-      <c r="H91" s="3"/>
-      <c r="I91" s="3"/>
-      <c r="J91" s="6"/>
-      <c r="K91" s="3"/>
-      <c r="L91" s="3"/>
-      <c r="M91" s="3"/>
-    </row>
-    <row r="92" spans="1:13" ht="15">
-      <c r="A92" s="3"/>
-      <c r="B92" s="3"/>
-      <c r="C92" s="3"/>
-      <c r="D92" s="3"/>
-      <c r="E92" s="3"/>
-      <c r="F92" s="3"/>
-      <c r="G92" s="3"/>
-      <c r="H92" s="3"/>
-      <c r="I92" s="3"/>
-      <c r="J92" s="6"/>
-      <c r="K92" s="3"/>
-      <c r="L92" s="3"/>
-      <c r="M92" s="3"/>
-    </row>
-    <row r="93" spans="1:13" ht="15">
-      <c r="A93" s="3"/>
-      <c r="B93" s="3"/>
-      <c r="C93" s="3"/>
-      <c r="D93" s="3"/>
-      <c r="E93" s="3"/>
-      <c r="F93" s="3"/>
-      <c r="G93" s="3"/>
-      <c r="H93" s="3"/>
-      <c r="I93" s="3"/>
-      <c r="J93" s="6"/>
-      <c r="K93" s="3"/>
-      <c r="L93" s="3"/>
-      <c r="M93" s="3"/>
-    </row>
-    <row r="94" spans="1:13" ht="15">
-      <c r="A94" s="3"/>
-      <c r="B94" s="3"/>
-      <c r="C94" s="3"/>
-      <c r="D94" s="3"/>
-      <c r="E94" s="3"/>
-      <c r="F94" s="3"/>
-      <c r="G94" s="3"/>
-      <c r="H94" s="3"/>
-      <c r="I94" s="3"/>
-      <c r="J94" s="6"/>
-      <c r="K94" s="3"/>
-      <c r="L94" s="3"/>
-      <c r="M94" s="3"/>
-    </row>
-    <row r="95" spans="1:13" ht="15">
-      <c r="A95" s="3"/>
-      <c r="B95" s="3"/>
-      <c r="C95" s="3"/>
-      <c r="D95" s="3"/>
-      <c r="E95" s="3"/>
-      <c r="F95" s="3"/>
-      <c r="G95" s="3"/>
-      <c r="H95" s="3"/>
-      <c r="I95" s="3"/>
-      <c r="J95" s="6"/>
-      <c r="K95" s="3"/>
-      <c r="L95" s="3"/>
-      <c r="M95" s="3"/>
-    </row>
-    <row r="96" spans="1:13" ht="15">
-      <c r="A96" s="3"/>
-      <c r="B96" s="3"/>
-      <c r="C96" s="3"/>
-      <c r="D96" s="3"/>
-      <c r="E96" s="3"/>
-      <c r="F96" s="3"/>
-      <c r="G96" s="3"/>
-      <c r="H96" s="3"/>
-      <c r="I96" s="3"/>
-      <c r="J96" s="6"/>
-      <c r="K96" s="3"/>
-      <c r="L96" s="3"/>
-      <c r="M96" s="3"/>
-    </row>
-    <row r="97" spans="1:13" ht="15">
-      <c r="A97" s="3"/>
-      <c r="B97" s="3"/>
-      <c r="C97" s="3"/>
-      <c r="D97" s="3"/>
-      <c r="E97" s="3"/>
-      <c r="F97" s="3"/>
-      <c r="G97" s="3"/>
-      <c r="H97" s="3"/>
-      <c r="I97" s="3"/>
-      <c r="J97" s="6"/>
-      <c r="K97" s="3"/>
-      <c r="L97" s="3"/>
-      <c r="M97" s="3"/>
-    </row>
-    <row r="98" spans="1:13" ht="15">
-      <c r="A98" s="3"/>
-      <c r="B98" s="3"/>
-      <c r="C98" s="3"/>
-      <c r="D98" s="3"/>
-      <c r="E98" s="3"/>
-      <c r="F98" s="3"/>
-      <c r="G98" s="3"/>
-      <c r="H98" s="3"/>
-      <c r="I98" s="3"/>
-      <c r="J98" s="6"/>
-      <c r="K98" s="3"/>
-      <c r="L98" s="3"/>
-      <c r="M98" s="3"/>
-    </row>
-    <row r="99" spans="1:13" ht="15">
-      <c r="A99" s="3"/>
-      <c r="B99" s="3"/>
-      <c r="C99" s="3"/>
-      <c r="D99" s="3"/>
-      <c r="E99" s="3"/>
-      <c r="F99" s="3"/>
-      <c r="G99" s="3"/>
-      <c r="H99" s="3"/>
-      <c r="I99" s="3"/>
-      <c r="J99" s="6"/>
-      <c r="K99" s="3"/>
-      <c r="L99" s="3"/>
-      <c r="M99" s="3"/>
-    </row>
-    <row r="100" spans="1:13" ht="15">
-      <c r="A100" s="3"/>
-      <c r="B100" s="3"/>
-      <c r="C100" s="3"/>
-      <c r="D100" s="3"/>
-      <c r="E100" s="3"/>
-      <c r="F100" s="3"/>
-      <c r="G100" s="3"/>
-      <c r="H100" s="3"/>
-      <c r="I100" s="3"/>
-      <c r="J100" s="6"/>
-      <c r="K100" s="3"/>
-      <c r="L100" s="3"/>
-      <c r="M100" s="3"/>
-    </row>
-    <row r="101" spans="1:13" ht="15">
-      <c r="A101" s="3"/>
-      <c r="B101" s="3"/>
-      <c r="C101" s="3"/>
-      <c r="D101" s="3"/>
-      <c r="E101" s="3"/>
-      <c r="F101" s="3"/>
-      <c r="G101" s="3"/>
-      <c r="H101" s="3"/>
-      <c r="I101" s="3"/>
-      <c r="J101" s="6"/>
-      <c r="K101" s="3"/>
-      <c r="L101" s="3"/>
-      <c r="M101" s="3"/>
-    </row>
-    <row r="102" spans="1:13" ht="15">
-      <c r="A102" s="3"/>
-      <c r="B102" s="3"/>
-      <c r="C102" s="3"/>
-      <c r="D102" s="3"/>
-      <c r="E102" s="3"/>
-      <c r="F102" s="3"/>
-      <c r="G102" s="3"/>
-      <c r="H102" s="3"/>
-      <c r="I102" s="3"/>
-      <c r="J102" s="6"/>
-      <c r="K102" s="3"/>
-      <c r="L102" s="3"/>
-      <c r="M102" s="3"/>
+    <row r="83" spans="1:13" ht="167.25">
+      <c r="A83" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" s="12" t="s">
+        <v>353</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F83" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="G83" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H83" t="s">
+        <v>30</v>
+      </c>
+      <c r="I83" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J83" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="K83" s="13" t="s">
+        <v>354</v>
+      </c>
+      <c r="L83" s="11" t="s">
+        <v>355</v>
+      </c>
+      <c r="M83" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" ht="213">
+      <c r="A84" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C84" s="12" t="s">
+        <v>356</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I84" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J84" s="6">
+        <v>46113</v>
+      </c>
+      <c r="K84" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="L84" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="M84" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" ht="167.25">
+      <c r="A85" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>359</v>
+      </c>
+      <c r="D85" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G85" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H85" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I85" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J85" s="6">
+        <v>45576</v>
+      </c>
+      <c r="K85" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="L85" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="M85" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" ht="183">
+      <c r="A86" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B86" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C86" s="12" t="s">
+        <v>362</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H86" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I86" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J86" s="6">
+        <v>46113</v>
+      </c>
+      <c r="K86" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="L86" s="11" t="s">
+        <v>364</v>
+      </c>
+      <c r="M86" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" ht="137.25">
+      <c r="A87" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C87" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="D87" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F87" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G87" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H87" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I87" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J87" s="6">
+        <v>46043</v>
+      </c>
+      <c r="K87" s="13" t="s">
+        <v>366</v>
+      </c>
+      <c r="L87" s="11" t="s">
+        <v>367</v>
+      </c>
+      <c r="M87" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" ht="198">
+      <c r="A88" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B88" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88" s="11" t="s">
+        <v>368</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F88" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G88" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I88" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J88" s="6">
+        <v>45870</v>
+      </c>
+      <c r="K88" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="L88" s="11" t="s">
+        <v>370</v>
+      </c>
+      <c r="M88" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="89" spans="1:13" ht="152.25">
+      <c r="A89" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C89" s="11" t="s">
+        <v>371</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F89" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H89" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I89" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J89" s="6">
+        <v>45689</v>
+      </c>
+      <c r="K89" s="13" t="s">
+        <v>372</v>
+      </c>
+      <c r="L89" s="11" t="s">
+        <v>373</v>
+      </c>
+      <c r="M89" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" ht="183">
+      <c r="A90" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C90" s="11" t="s">
+        <v>374</v>
+      </c>
+      <c r="D90" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F90" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H90" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I90" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J90" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K90" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="L90" s="11" t="s">
+        <v>376</v>
+      </c>
+      <c r="M90" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="91" spans="1:13" ht="213">
+      <c r="A91" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="D91" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F91" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G91" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H91" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I91" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J91" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K91" s="13" t="s">
+        <v>378</v>
+      </c>
+      <c r="L91" s="11" t="s">
+        <v>379</v>
+      </c>
+      <c r="M91" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" ht="121.5">
+      <c r="A92" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C92" s="11" t="s">
+        <v>380</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F92" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G92" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H92" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I92" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J92" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="K92" s="13" t="s">
+        <v>382</v>
+      </c>
+      <c r="L92" s="11" t="s">
+        <v>383</v>
+      </c>
+      <c r="M92" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="93" spans="1:13" ht="91.5">
+      <c r="A93" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C93" s="11" t="s">
+        <v>384</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F93" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="G93" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H93" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I93" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J93" s="6">
+        <v>45748</v>
+      </c>
+      <c r="K93" s="13" t="s">
+        <v>385</v>
+      </c>
+      <c r="L93" s="11" t="s">
+        <v>386</v>
+      </c>
+      <c r="M93" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="94" spans="1:13" ht="198">
+      <c r="A94" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C94" s="11" t="s">
+        <v>387</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E94" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F94" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G94" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H94" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I94" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J94" t="s">
+        <v>388</v>
+      </c>
+      <c r="K94" s="13" t="s">
+        <v>389</v>
+      </c>
+      <c r="L94" s="11" t="s">
+        <v>390</v>
+      </c>
+      <c r="M94" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="95" spans="1:13" ht="137.25">
+      <c r="A95" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C95" s="11" t="s">
+        <v>391</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E95" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F95" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G95" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H95" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I95" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J95" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="K95" s="13" t="s">
+        <v>392</v>
+      </c>
+      <c r="L95" s="12" t="s">
+        <v>393</v>
+      </c>
+      <c r="M95" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="96" spans="1:13" ht="76.5">
+      <c r="A96" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C96" s="11" t="s">
+        <v>394</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E96" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F96" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G96" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H96" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I96" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J96" s="14">
+        <v>45663</v>
+      </c>
+      <c r="K96" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="L96" s="12" t="s">
+        <v>395</v>
+      </c>
+      <c r="M96" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13" ht="121.5">
+      <c r="A97" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C97" s="11" t="s">
+        <v>396</v>
+      </c>
+      <c r="D97" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F97" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G97" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H97" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I97" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J97" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="K97" s="13" t="s">
+        <v>397</v>
+      </c>
+      <c r="L97" s="12" t="s">
+        <v>398</v>
+      </c>
+      <c r="M97" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13" ht="183">
+      <c r="A98" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C98" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="D98" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="E98" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F98" t="s">
+        <v>400</v>
+      </c>
+      <c r="G98" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H98" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I98" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J98" s="14">
+        <v>45660</v>
+      </c>
+      <c r="K98" s="13" t="s">
+        <v>401</v>
+      </c>
+      <c r="L98" s="12" t="s">
+        <v>402</v>
+      </c>
+      <c r="M98" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13" ht="183">
+      <c r="A99" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C99" s="11" t="s">
+        <v>403</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F99" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G99" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H99" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J99" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="K99" s="13" t="s">
+        <v>404</v>
+      </c>
+      <c r="L99" s="11" t="s">
+        <v>405</v>
+      </c>
+      <c r="M99" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="100" spans="1:13" ht="152.25">
+      <c r="A100" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C100" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D100" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F100" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="G100" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H100" t="s">
+        <v>30</v>
+      </c>
+      <c r="I100" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J100" s="6">
+        <v>45200</v>
+      </c>
+      <c r="K100" s="13" t="s">
+        <v>407</v>
+      </c>
+      <c r="L100" s="12" t="s">
+        <v>408</v>
+      </c>
+      <c r="M100" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" ht="121.5">
+      <c r="A101" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C101" s="15" t="s">
+        <v>409</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F101" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="G101" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H101" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I101" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J101" s="6">
+        <v>45292</v>
+      </c>
+      <c r="K101" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="L101" s="15" t="s">
+        <v>410</v>
+      </c>
+      <c r="M101" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="102" spans="1:13" ht="30.75">
+      <c r="A102" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D102" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F102" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="G102" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H102" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I102" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J102" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K102" s="13" t="s">
+        <v>413</v>
+      </c>
+      <c r="L102" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="M102" s="3" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="103" spans="1:13" ht="15">
-      <c r="A103" s="3"/>
-      <c r="B103" s="3"/>
-      <c r="C103" s="3"/>
-      <c r="D103" s="3"/>
-      <c r="E103" s="3"/>
-      <c r="F103" s="3"/>
-      <c r="G103" s="3"/>
-      <c r="H103" s="3"/>
-      <c r="I103" s="3"/>
-      <c r="J103" s="6"/>
-      <c r="K103" s="3"/>
-      <c r="L103" s="3"/>
-      <c r="M103" s="3"/>
-    </row>
-    <row r="104" spans="1:13" ht="15">
-      <c r="A104" s="3"/>
-      <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
-      <c r="D104" s="3"/>
-      <c r="E104" s="3"/>
-      <c r="F104" s="3"/>
-      <c r="G104" s="3"/>
-      <c r="H104" s="3"/>
-      <c r="I104" s="3"/>
-      <c r="J104" s="6"/>
-      <c r="K104" s="3"/>
-      <c r="L104" s="3"/>
-      <c r="M104" s="3"/>
-    </row>
-    <row r="105" spans="1:13" ht="15"/>
-    <row r="106" spans="1:13" ht="15"/>
+      <c r="A103" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F103" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="G103" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H103" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I103" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J103" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K103" s="13" t="s">
+        <v>418</v>
+      </c>
+      <c r="L103" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="M103" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="104" spans="1:13" ht="30.75">
+      <c r="A104" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="D104" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F104" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="G104" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H104" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I104" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J104" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K104" s="13" t="s">
+        <v>422</v>
+      </c>
+      <c r="L104" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="M104" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="105" spans="1:13" ht="15">
+      <c r="A105" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>424</v>
+      </c>
+      <c r="D105" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F105" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="G105" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H105" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I105" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J105" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="K105" s="13" t="s">
+        <v>426</v>
+      </c>
+      <c r="L105" s="3" t="s">
+        <v>427</v>
+      </c>
+      <c r="M105" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="106" spans="1:13" ht="15">
+      <c r="A106" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F106" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="G106" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H106" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I106" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J106" s="6" t="s">
+        <v>430</v>
+      </c>
+      <c r="K106" s="13" t="s">
+        <v>431</v>
+      </c>
+      <c r="L106" s="3" t="s">
+        <v>432</v>
+      </c>
+      <c r="M106" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="107" spans="1:13" ht="15">
+      <c r="A107" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F107" s="3" t="s">
+        <v>434</v>
+      </c>
+      <c r="G107" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H107" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I107" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="J107" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="K107" s="13" t="s">
+        <v>437</v>
+      </c>
+      <c r="L107" s="3" t="s">
+        <v>438</v>
+      </c>
+      <c r="M107" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="108" spans="1:13" ht="30.75">
+      <c r="A108" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="D108" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F108" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H108" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I108" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J108" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K108" s="13" t="s">
+        <v>441</v>
+      </c>
+      <c r="L108" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="M108" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="109" spans="1:13" ht="30.75">
+      <c r="A109" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>443</v>
+      </c>
+      <c r="D109" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F109" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H109" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I109" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J109" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="K109" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="L109" s="3" t="s">
+        <v>446</v>
+      </c>
+      <c r="M109" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="110" spans="1:13" ht="30.75">
+      <c r="A110" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="D110" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E110" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F110" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="G110" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H110" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I110" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J110" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="K110" s="13" t="s">
+        <v>449</v>
+      </c>
+      <c r="L110" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="M110" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="111" spans="1:13" ht="15">
+      <c r="A111" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F111" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="G111" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H111" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I111" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J111" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K111" s="13" t="s">
+        <v>453</v>
+      </c>
+      <c r="L111" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="M111" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="112" spans="1:13" ht="30.75">
+      <c r="A112" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>455</v>
+      </c>
+      <c r="D112" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E112" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F112" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="G112" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H112" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I112" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J112" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K112" s="13" t="s">
+        <v>457</v>
+      </c>
+      <c r="L112" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="M112" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="113" spans="1:13" ht="30.75">
+      <c r="A113" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C113" s="3" t="s">
+        <v>459</v>
+      </c>
+      <c r="D113" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="E113" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F113" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="G113" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H113" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I113" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J113" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K113" s="13" t="s">
+        <v>460</v>
+      </c>
+      <c r="L113" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="M113" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="114" spans="1:13" ht="30.75">
+      <c r="A114" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C114" s="3" t="s">
+        <v>462</v>
+      </c>
+      <c r="D114" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F114" s="3" t="s">
+        <v>463</v>
+      </c>
+      <c r="G114" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H114" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I114" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J114" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K114" s="13" t="s">
+        <v>464</v>
+      </c>
+      <c r="L114" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="M114" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="115" spans="1:13" ht="15">
+      <c r="A115" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E115" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F115" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="G115" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H115" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I115" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J115" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K115" s="13" t="s">
+        <v>468</v>
+      </c>
+      <c r="L115" s="3" t="s">
+        <v>469</v>
+      </c>
+      <c r="M115" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="116" spans="1:13" ht="15">
+      <c r="A116" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E116" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F116" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="G116" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H116" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I116" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J116" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="K116" s="13" t="s">
+        <v>473</v>
+      </c>
+      <c r="L116" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="M116" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="117" spans="1:13" ht="30.75">
+      <c r="A117" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="D117" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E117" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F117" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="G117" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H117" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I117" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="J117" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K117" s="13" t="s">
+        <v>477</v>
+      </c>
+      <c r="L117" s="3" t="s">
+        <v>478</v>
+      </c>
+      <c r="M117" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="118" spans="1:13" ht="30.75">
+      <c r="A118" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>479</v>
+      </c>
+      <c r="D118" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E118" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F118" s="3" t="s">
+        <v>480</v>
+      </c>
+      <c r="G118" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H118" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I118" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J118" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="K118" s="13" t="s">
+        <v>482</v>
+      </c>
+      <c r="L118" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="M118" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="119" spans="1:13" ht="30.75">
+      <c r="A119" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="D119" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F119" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G119" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H119" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I119" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J119" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K119" s="13" t="s">
+        <v>485</v>
+      </c>
+      <c r="L119" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="M119" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="120" spans="1:13" ht="30.75">
+      <c r="A120" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="D120" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E120" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F120" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H120" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I120" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="J120" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K120" s="13" t="s">
+        <v>489</v>
+      </c>
+      <c r="L120" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="M120" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="121" spans="1:13" ht="15">
+      <c r="A121" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="D121" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E121" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F121" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="G121" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H121" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I121" s="3" t="s">
+        <v>435</v>
+      </c>
+      <c r="J121" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="K121" s="13" t="s">
+        <v>493</v>
+      </c>
+      <c r="L121" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="M121" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="122" spans="1:13">
+      <c r="A122" s="3"/>
+      <c r="B122" s="3"/>
+      <c r="C122" s="3"/>
+      <c r="D122" s="3"/>
+      <c r="E122" s="3"/>
+      <c r="F122" s="3"/>
+      <c r="G122" s="3"/>
+      <c r="H122" s="3"/>
+      <c r="I122" s="3"/>
+      <c r="J122" s="6"/>
+      <c r="K122" s="3"/>
+      <c r="L122" s="3"/>
+      <c r="M122" s="3"/>
+    </row>
+    <row r="123" spans="1:13">
+      <c r="A123" s="3"/>
+      <c r="B123" s="3"/>
+      <c r="C123" s="3"/>
+      <c r="D123" s="3"/>
+      <c r="E123" s="3"/>
+      <c r="F123" s="3"/>
+      <c r="G123" s="3"/>
+      <c r="H123" s="3"/>
+      <c r="I123" s="3"/>
+      <c r="J123" s="6"/>
+      <c r="K123" s="3"/>
+      <c r="L123" s="3"/>
+      <c r="M123" s="3"/>
+    </row>
+    <row r="124" spans="1:13">
+      <c r="A124" s="3"/>
+      <c r="B124" s="3"/>
+      <c r="C124" s="3"/>
+      <c r="D124" s="3"/>
+      <c r="E124" s="3"/>
+      <c r="F124" s="3"/>
+      <c r="G124" s="3"/>
+      <c r="H124" s="3"/>
+      <c r="I124" s="3"/>
+      <c r="J124" s="6"/>
+      <c r="K124" s="3"/>
+      <c r="L124" s="3"/>
+      <c r="M124" s="3"/>
+    </row>
+    <row r="125" spans="1:13">
+      <c r="A125" s="3"/>
+      <c r="B125" s="3"/>
+      <c r="C125" s="3"/>
+      <c r="D125" s="3"/>
+      <c r="E125" s="3"/>
+      <c r="F125" s="3"/>
+      <c r="G125" s="3"/>
+      <c r="H125" s="3"/>
+      <c r="I125" s="3"/>
+      <c r="J125" s="6"/>
+      <c r="K125" s="3"/>
+      <c r="L125" s="3"/>
+      <c r="M125" s="3"/>
+    </row>
+    <row r="126" spans="1:13">
+      <c r="A126" s="3"/>
+      <c r="B126" s="3"/>
+      <c r="C126" s="3"/>
+      <c r="D126" s="3"/>
+      <c r="E126" s="3"/>
+      <c r="F126" s="3"/>
+      <c r="G126" s="3"/>
+      <c r="H126" s="3"/>
+      <c r="I126" s="3"/>
+      <c r="J126" s="6"/>
+      <c r="K126" s="3"/>
+      <c r="L126" s="3"/>
+      <c r="M126" s="3"/>
+    </row>
+    <row r="127" spans="1:13">
+      <c r="A127" s="3"/>
+      <c r="B127" s="3"/>
+      <c r="C127" s="3"/>
+      <c r="D127" s="3"/>
+      <c r="E127" s="3"/>
+      <c r="F127" s="3"/>
+      <c r="G127" s="3"/>
+      <c r="H127" s="3"/>
+      <c r="I127" s="3"/>
+      <c r="J127" s="6"/>
+      <c r="K127" s="3"/>
+      <c r="L127" s="3"/>
+      <c r="M127" s="3"/>
+    </row>
+    <row r="128" spans="1:13">
+      <c r="A128" s="3"/>
+      <c r="B128" s="3"/>
+      <c r="C128" s="3"/>
+      <c r="D128" s="3"/>
+      <c r="E128" s="3"/>
+      <c r="F128" s="3"/>
+      <c r="G128" s="3"/>
+      <c r="H128" s="3"/>
+      <c r="I128" s="3"/>
+      <c r="J128" s="6"/>
+      <c r="K128" s="3"/>
+      <c r="L128" s="3"/>
+      <c r="M128" s="3"/>
+    </row>
+    <row r="129" spans="1:13">
+      <c r="A129" s="3"/>
+      <c r="B129" s="3"/>
+      <c r="C129" s="3"/>
+      <c r="D129" s="3"/>
+      <c r="E129" s="3"/>
+      <c r="F129" s="3"/>
+      <c r="G129" s="3"/>
+      <c r="H129" s="3"/>
+      <c r="I129" s="3"/>
+      <c r="J129" s="6"/>
+      <c r="K129" s="3"/>
+      <c r="L129" s="3"/>
+      <c r="M129" s="3"/>
+    </row>
+    <row r="130" spans="1:13">
+      <c r="A130" s="3"/>
+      <c r="B130" s="3"/>
+      <c r="C130" s="3"/>
+      <c r="D130" s="3"/>
+      <c r="E130" s="3"/>
+      <c r="F130" s="3"/>
+      <c r="G130" s="3"/>
+      <c r="H130" s="3"/>
+      <c r="I130" s="3"/>
+      <c r="J130" s="6"/>
+      <c r="K130" s="3"/>
+      <c r="L130" s="3"/>
+      <c r="M130" s="3"/>
+    </row>
+    <row r="131" spans="1:13">
+      <c r="A131" s="3"/>
+      <c r="B131" s="3"/>
+      <c r="C131" s="3"/>
+      <c r="D131" s="3"/>
+      <c r="E131" s="3"/>
+      <c r="F131" s="3"/>
+      <c r="G131" s="3"/>
+      <c r="H131" s="3"/>
+      <c r="I131" s="3"/>
+      <c r="J131" s="6"/>
+      <c r="K131" s="3"/>
+      <c r="L131" s="3"/>
+      <c r="M131" s="3"/>
+    </row>
+    <row r="132" spans="1:13">
+      <c r="A132" s="3"/>
+      <c r="B132" s="3"/>
+      <c r="C132" s="3"/>
+      <c r="D132" s="3"/>
+      <c r="E132" s="3"/>
+      <c r="F132" s="3"/>
+      <c r="G132" s="3"/>
+      <c r="H132" s="3"/>
+      <c r="I132" s="3"/>
+      <c r="J132" s="6"/>
+      <c r="K132" s="3"/>
+      <c r="L132" s="3"/>
+      <c r="M132" s="3"/>
+    </row>
+    <row r="133" spans="1:13">
+      <c r="A133" s="3"/>
+      <c r="B133" s="3"/>
+      <c r="C133" s="3"/>
+      <c r="D133" s="3"/>
+      <c r="E133" s="3"/>
+      <c r="F133" s="3"/>
+      <c r="G133" s="3"/>
+      <c r="H133" s="3"/>
+      <c r="I133" s="3"/>
+      <c r="J133" s="6"/>
+      <c r="K133" s="3"/>
+      <c r="L133" s="3"/>
+      <c r="M133" s="3"/>
+    </row>
+    <row r="134" spans="1:13">
+      <c r="A134" s="3"/>
+      <c r="B134" s="3"/>
+      <c r="C134" s="3"/>
+      <c r="D134" s="3"/>
+      <c r="E134" s="3"/>
+      <c r="F134" s="3"/>
+      <c r="G134" s="3"/>
+      <c r="H134" s="3"/>
+      <c r="I134" s="3"/>
+      <c r="J134" s="6"/>
+      <c r="K134" s="3"/>
+      <c r="L134" s="3"/>
+      <c r="M134" s="3"/>
+    </row>
+    <row r="135" spans="1:13">
+      <c r="A135" s="3"/>
+      <c r="B135" s="3"/>
+      <c r="C135" s="3"/>
+      <c r="D135" s="3"/>
+      <c r="E135" s="3"/>
+      <c r="F135" s="3"/>
+      <c r="G135" s="3"/>
+      <c r="H135" s="3"/>
+      <c r="I135" s="3"/>
+      <c r="J135" s="6"/>
+      <c r="K135" s="3"/>
+      <c r="L135" s="3"/>
+      <c r="M135" s="3"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation allowBlank="1" sqref="G1:H1" xr:uid="{368EE41E-2705-1B43-9A52-5A9881088DDE}"/>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="K83" r:id="rId1" xr:uid="{B26B418E-DD48-4E83-BB37-848152B687EC}"/>
+    <hyperlink ref="K84" r:id="rId2" xr:uid="{6C54A787-4172-4FAF-8153-0DAC9DCDB938}"/>
+    <hyperlink ref="K85" r:id="rId3" xr:uid="{4FBB6745-680C-4EF0-B8E7-1B954BB30B4E}"/>
+    <hyperlink ref="K86" r:id="rId4" xr:uid="{D46786CB-5B8E-4706-9F2B-4C0AD8E73B27}"/>
+    <hyperlink ref="K87" r:id="rId5" xr:uid="{657351BD-88E6-4A80-AB85-9068838CB91A}"/>
+    <hyperlink ref="K88" r:id="rId6" xr:uid="{CE41647C-65AC-4023-85FE-FB3A4CBE66D1}"/>
+    <hyperlink ref="K89" r:id="rId7" xr:uid="{41B93F60-8676-42F8-AB3B-0EF536AA7128}"/>
+    <hyperlink ref="K90" r:id="rId8" xr:uid="{7CC0DEF0-305F-42A6-ABCE-F1487F0EC1DB}"/>
+    <hyperlink ref="K91" r:id="rId9" xr:uid="{75413EF0-9D07-47AC-B005-88AA88E02B09}"/>
+    <hyperlink ref="K92" r:id="rId10" xr:uid="{46EE40CD-1B55-45EE-B796-ADB3AB578548}"/>
+    <hyperlink ref="K93" r:id="rId11" xr:uid="{0FA44BBB-5B41-469E-AC62-F410BFB96E6F}"/>
+    <hyperlink ref="K94" r:id="rId12" xr:uid="{7948EF90-CF8A-4D88-9A7E-76F9DF4CAC33}"/>
+    <hyperlink ref="K95" r:id="rId13" xr:uid="{7D91FB46-A739-499A-B86B-C5C786D36D80}"/>
+    <hyperlink ref="K96" r:id="rId14" xr:uid="{78008A78-AB32-4432-8076-BF165A896490}"/>
+    <hyperlink ref="K97" r:id="rId15" xr:uid="{2109B0C5-5EF4-4DA8-8534-E6A839219026}"/>
+    <hyperlink ref="K98" r:id="rId16" xr:uid="{DE1111F3-01B3-4EE7-971F-3DA2E7AC2683}"/>
+    <hyperlink ref="K99" r:id="rId17" xr:uid="{52E86ECD-12AB-4255-8975-CF40CABAB84F}"/>
+    <hyperlink ref="K100" r:id="rId18" xr:uid="{6C0845F7-D950-4600-A5A4-D3EC5EC18203}"/>
+    <hyperlink ref="K101" r:id="rId19" xr:uid="{30A5C176-4E69-4953-90F1-7D8FD8B8AB96}"/>
+    <hyperlink ref="K102" r:id="rId20" xr:uid="{528CA009-5514-4DB0-BBA7-E8F8FD6113CB}"/>
+    <hyperlink ref="K103" r:id="rId21" xr:uid="{1591B514-C960-482D-B88C-727F4B4D28CC}"/>
+    <hyperlink ref="K104" r:id="rId22" xr:uid="{41CF9F50-2D43-4ADE-BC9E-B7DEE42E292B}"/>
+    <hyperlink ref="K105" r:id="rId23" xr:uid="{73133CAA-A759-429E-B124-8D3B9B1B35BF}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId24"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
@@ -5383,13 +7326,13 @@
           <x14:formula1>
             <xm:f>'Vinculo con educacion'!$A$1:$A$2</xm:f>
           </x14:formula1>
-          <xm:sqref>H84:H1048576 H2:H82</xm:sqref>
+          <xm:sqref>H2:H82 H84:H1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CB47FA5A-6567-2547-B57E-466B59F1912C}">
           <x14:formula1>
             <xm:f>'Tipo de norma'!$A$1:$A$10</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D1048576</xm:sqref>
+          <xm:sqref>D2:D109 D111:D1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{EF828923-8993-5646-A9D3-B4E6E4049B2E}">
           <x14:formula1>
@@ -5437,7 +7380,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.6">
       <c r="A1" s="1" t="s">
-        <v>353</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="15.6">
@@ -5447,157 +7390,157 @@
     </row>
     <row r="3" spans="1:1" ht="15.6">
       <c r="A3" s="1" t="s">
-        <v>354</v>
+        <v>496</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="15.6">
       <c r="A4" s="1" t="s">
-        <v>355</v>
+        <v>497</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="15.6">
       <c r="A5" s="1" t="s">
-        <v>356</v>
+        <v>498</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="15.6">
       <c r="A6" s="1" t="s">
-        <v>357</v>
+        <v>499</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="15.6">
       <c r="A7" s="1" t="s">
-        <v>358</v>
+        <v>500</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="15.6">
       <c r="A8" s="1" t="s">
-        <v>359</v>
+        <v>501</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.6">
       <c r="A9" s="1" t="s">
-        <v>360</v>
+        <v>502</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="15.6">
       <c r="A10" s="1" t="s">
-        <v>361</v>
+        <v>503</v>
       </c>
     </row>
     <row r="11" spans="1:1" ht="15.6">
       <c r="A11" s="1" t="s">
-        <v>362</v>
+        <v>504</v>
       </c>
     </row>
     <row r="12" spans="1:1" ht="15.6">
       <c r="A12" s="1" t="s">
-        <v>363</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" spans="1:1" ht="15.6">
       <c r="A13" s="1" t="s">
-        <v>364</v>
+        <v>506</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="15.6">
       <c r="A14" s="1" t="s">
-        <v>365</v>
+        <v>507</v>
       </c>
     </row>
     <row r="15" spans="1:1" ht="15.6">
       <c r="A15" s="1" t="s">
-        <v>366</v>
+        <v>508</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="15.6">
       <c r="A16" s="1" t="s">
-        <v>367</v>
+        <v>509</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="15.6">
       <c r="A17" s="1" t="s">
-        <v>368</v>
+        <v>510</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15.6">
       <c r="A18" s="1" t="s">
-        <v>369</v>
+        <v>511</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="15.6">
       <c r="A19" s="1" t="s">
-        <v>370</v>
+        <v>512</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15.6">
       <c r="A20" s="1" t="s">
-        <v>371</v>
+        <v>513</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="15.6">
       <c r="A21" s="1" t="s">
-        <v>372</v>
+        <v>514</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="15.6">
       <c r="A22" s="1" t="s">
-        <v>373</v>
+        <v>515</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="15.6">
       <c r="A23" s="1" t="s">
-        <v>374</v>
+        <v>516</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="15.6">
       <c r="A24" s="1" t="s">
-        <v>375</v>
+        <v>517</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="15.6">
       <c r="A25" s="1" t="s">
-        <v>376</v>
+        <v>518</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="15.6">
       <c r="A26" s="1" t="s">
-        <v>377</v>
+        <v>519</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="15.6">
       <c r="A27" s="1" t="s">
-        <v>378</v>
+        <v>520</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="15.6">
       <c r="A28" s="1" t="s">
-        <v>379</v>
+        <v>521</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="15.6">
       <c r="A29" s="1" t="s">
-        <v>380</v>
+        <v>522</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="15.6">
       <c r="A30" s="1" t="s">
-        <v>381</v>
+        <v>523</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="15.6">
       <c r="A31" s="1" t="s">
-        <v>382</v>
+        <v>524</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="15.6">
       <c r="A32" s="1" t="s">
-        <v>383</v>
+        <v>525</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="15.6">
       <c r="A33" s="1" t="s">
-        <v>384</v>
+        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -5618,7 +7561,7 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>385</v>
+        <v>527</v>
       </c>
     </row>
     <row r="3" spans="1:1">
@@ -5687,7 +7630,7 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>386</v>
+        <v>528</v>
       </c>
     </row>
   </sheetData>
@@ -5773,7 +7716,7 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>387</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4" spans="1:1">

</xml_diff>